<commit_message>
auto: update dashboard report and AI map
</commit_message>
<xml_diff>
--- a/data/typhoon_predictions.xlsx
+++ b/data/typhoon_predictions.xlsx
@@ -495,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>13.3</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -517,13 +517,13 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>33.3</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5">
@@ -539,13 +539,13 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="6">
@@ -567,7 +567,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>1.3</v>
       </c>
       <c r="F7" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="8">
@@ -599,19 +599,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>16</v>
+        <v>5.3</v>
       </c>
       <c r="D8" t="n">
         <v>25.3</v>
       </c>
       <c r="E8" t="n">
-        <v>9.300000000000001</v>
+        <v>2.7</v>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="9">
@@ -630,10 +630,10 @@
         <v>38.7</v>
       </c>
       <c r="E9" t="n">
-        <v>29.3</v>
+        <v>28</v>
       </c>
       <c r="F9" t="n">
-        <v>9.9</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="10">
@@ -652,10 +652,10 @@
         <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>40</v>
+        <v>38.7</v>
       </c>
       <c r="F10" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -677,7 +677,7 @@
         <v>38.7</v>
       </c>
       <c r="F11" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="12">
@@ -712,16 +712,16 @@
         <v>13.3</v>
       </c>
       <c r="C13" t="n">
-        <v>34.7</v>
+        <v>32</v>
       </c>
       <c r="D13" t="n">
         <v>13.3</v>
       </c>
       <c r="E13" t="n">
-        <v>13.3</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -734,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>16</v>
+        <v>14.7</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="15">
@@ -831,7 +831,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">

</xml_diff>